<commit_message>
correct xlsx for symbol
</commit_message>
<xml_diff>
--- a/db/hwdb/А004.xlsx
+++ b/db/hwdb/А004.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="28260" windowHeight="12360"/>
+    <workbookView xWindow="120" yWindow="105" windowWidth="28260" windowHeight="12360" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Controls" sheetId="4" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="166">
   <si>
     <t>Modbus RTU</t>
   </si>
@@ -687,7 +687,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -861,6 +861,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -68212,8 +68215,8 @@
       </c>
       <c r="V12" s="47"/>
       <c r="W12" s="47"/>
-      <c r="X12" s="47">
-        <v>0</v>
+      <c r="X12" s="62" t="s">
+        <v>53</v>
       </c>
       <c r="Y12" s="47">
         <v>0</v>
@@ -68274,7 +68277,7 @@
       <c r="BF12" s="53"/>
       <c r="BG12" s="54" t="str">
         <f t="shared" si="4"/>
-        <v>description: "Имя сигнала для отображения в схемах 1", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: 0, eventRegistration: 0</v>
+        <v>description: "Имя сигнала для отображения в схемах 1", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: null, eventRegistration: 0</v>
       </c>
     </row>
     <row r="13" spans="1:16379" s="39" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -69595,8 +69598,8 @@
       </c>
       <c r="V22" s="25"/>
       <c r="W22" s="25"/>
-      <c r="X22" s="25">
-        <v>0</v>
+      <c r="X22" s="62" t="s">
+        <v>53</v>
       </c>
       <c r="Y22" s="25">
         <v>0</v>
@@ -69657,7 +69660,7 @@
       <c r="BF22" s="23"/>
       <c r="BG22" s="21" t="str">
         <f t="shared" si="4"/>
-        <v>description: "Имя сигнала для отображения в схемах 2", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: 0, eventRegistration: 0</v>
+        <v>description: "Имя сигнала для отображения в схемах 2", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: null, eventRegistration: 0</v>
       </c>
     </row>
     <row r="23" spans="1:59" s="55" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -70978,8 +70981,8 @@
       </c>
       <c r="V32" s="47"/>
       <c r="W32" s="47"/>
-      <c r="X32" s="47">
-        <v>0</v>
+      <c r="X32" s="62" t="s">
+        <v>53</v>
       </c>
       <c r="Y32" s="47">
         <v>0</v>
@@ -71040,7 +71043,7 @@
       <c r="BF32" s="53"/>
       <c r="BG32" s="54" t="str">
         <f t="shared" si="4"/>
-        <v>description: "Имя сигнала для отображения в схемах 3", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: 0, eventRegistration: 0</v>
+        <v>description: "Имя сигнала для отображения в схемах 3", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: null, eventRegistration: 0</v>
       </c>
     </row>
     <row r="33" spans="1:59" s="39" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -72361,8 +72364,8 @@
       </c>
       <c r="V42" s="25"/>
       <c r="W42" s="25"/>
-      <c r="X42" s="25">
-        <v>0</v>
+      <c r="X42" s="62" t="s">
+        <v>53</v>
       </c>
       <c r="Y42" s="25">
         <v>0</v>
@@ -72423,7 +72426,7 @@
       <c r="BF42" s="23"/>
       <c r="BG42" s="21" t="str">
         <f t="shared" si="4"/>
-        <v>description: "Имя сигнала для отображения в схемах 4", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: 0, eventRegistration: 0</v>
+        <v>description: "Имя сигнала для отображения в схемах 4", note: "Пользовательское имя сигнала для отображения", group: "setting", minValue: 0, maxValue: 99, step: 1, units: "Символ", defaultValue: null, eventRegistration: 0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>